<commit_message>
Dashboard update Fri 07/31/2026 13:07
</commit_message>
<xml_diff>
--- a/data/Lease Builder/MSP_Key_Provisions Template.xlsx
+++ b/data/Lease Builder/MSP_Key_Provisions Template.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\Lease Builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BE04CA6-C653-4505-88AB-ED14802844C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9527B21-648B-433D-86CC-B10355BFD7A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Key Provisions" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Key Provisions'!$A$1:$G$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Key Provisions'!$A$1:$Q$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="110">
   <si>
     <t>Group</t>
   </si>
@@ -47,6 +47,9 @@
     <t>Key Provision</t>
   </si>
   <si>
+    <t>Current Value</t>
+  </si>
+  <si>
     <t>Link</t>
   </si>
   <si>
@@ -56,18 +59,60 @@
     <t>Bookmark</t>
   </si>
   <si>
+    <t>Alt 1</t>
+  </si>
+  <si>
+    <t>Alt 2</t>
+  </si>
+  <si>
+    <t>Alt 3</t>
+  </si>
+  <si>
+    <t>Alt 4</t>
+  </si>
+  <si>
+    <t>Alt 5</t>
+  </si>
+  <si>
+    <t>Alt 6</t>
+  </si>
+  <si>
+    <t>Alt 7</t>
+  </si>
+  <si>
+    <t>Alt 8</t>
+  </si>
+  <si>
+    <t>Alt 9</t>
+  </si>
+  <si>
+    <t>Alt 10</t>
+  </si>
+  <si>
     <t>Mandatory</t>
   </si>
   <si>
     <t>Property</t>
   </si>
   <si>
+    <t>114 Central Ave (also known as 102-104 Quimby St), Westfield, NJ 07090</t>
+  </si>
+  <si>
     <t>Section 1 — Premises</t>
   </si>
   <si>
     <t>Tx_BuildingAddress</t>
   </si>
   <si>
+    <t>1280 Springfield</t>
+  </si>
+  <si>
+    <t>15 South Street</t>
+  </si>
+  <si>
+    <t>36 South Street</t>
+  </si>
+  <si>
     <t>Lease Execution Date</t>
   </si>
   <si>
@@ -321,33 +366,6 @@
   </si>
   <si>
     <t>Tx_LandlordContFitUp</t>
-  </si>
-  <si>
-    <t>Current Value</t>
-  </si>
-  <si>
-    <t>114 Central Ave (also known as 102-104 Quimby St), Westfield, NJ 07090</t>
-  </si>
-  <si>
-    <t>Alt 1</t>
-  </si>
-  <si>
-    <t>Alt 2</t>
-  </si>
-  <si>
-    <t>Alt 3</t>
-  </si>
-  <si>
-    <t>Alt 4</t>
-  </si>
-  <si>
-    <t>1280 Springfield</t>
-  </si>
-  <si>
-    <t>15 South Street</t>
-  </si>
-  <si>
-    <t>36 South Street</t>
   </si>
 </sst>
 </file>
@@ -687,7 +705,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -697,10 +715,9 @@
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="6" max="6" width="34" customWidth="1"/>
     <col min="7" max="7" width="13" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="65.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -711,642 +728,660 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>97</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>99</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B2" t="b">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
+        <v>19</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>96</v>
+        <v>19</v>
       </c>
       <c r="I2" t="s">
-        <v>101</v>
+        <v>22</v>
       </c>
       <c r="J2" t="s">
-        <v>102</v>
+        <v>23</v>
       </c>
       <c r="K2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B3" t="b">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
       </c>
       <c r="F3" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B4" t="b">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B5" t="b">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B6" t="b">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
         <v>20</v>
       </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
-        <v>8</v>
-      </c>
       <c r="G6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B7" t="b">
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B8" t="b">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B9" t="b">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B10" t="b">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B11" t="b">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B12" t="b">
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G12" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B13" t="b">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G13" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B14" t="b">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="G14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B15" t="b">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="G15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B16" t="b">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B17" t="b">
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="G17" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B18" t="b">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="D18" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
       </c>
       <c r="F18" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G18" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B19" t="b">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="G19" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B20" t="b">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="D20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" t="s">
         <v>66</v>
       </c>
-      <c r="E20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F20" t="s">
-        <v>51</v>
-      </c>
       <c r="G20" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B21" t="b">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="D21" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="G21" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B22" t="b">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="D22" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="G22" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B23" t="b">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="D23" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G23" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B24" t="b">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="D24" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="E24" t="b">
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="G24" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B25" t="b">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="D25" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="E25" t="b">
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="G25" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B26" t="b">
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="E26" t="b">
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="G26" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B27" t="b">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="D27" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="E27" t="b">
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="G27" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G27" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:Q27" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dashboard update Fri 07/31/2026 13:16
</commit_message>
<xml_diff>
--- a/data/Lease Builder/MSP_Key_Provisions Template.xlsx
+++ b/data/Lease Builder/MSP_Key_Provisions Template.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\Lease Builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9527B21-648B-433D-86CC-B10355BFD7A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE750ABC-9AE6-486A-8B46-32D2474091DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5070" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Key Provisions" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Key Provisions'!$A$1:$Q$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Key Provisions'!$A$1:$R$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="108">
   <si>
     <t>Group</t>
   </si>
@@ -50,6 +50,9 @@
     <t>Current Value</t>
   </si>
   <si>
+    <t>Use Choice</t>
+  </si>
+  <si>
     <t>Link</t>
   </si>
   <si>
@@ -95,7 +98,7 @@
     <t>Property</t>
   </si>
   <si>
-    <t>114 Central Ave (also known as 102-104 Quimby St), Westfield, NJ 07090</t>
+    <t>1280</t>
   </si>
   <si>
     <t>Section 1 — Premises</t>
@@ -104,15 +107,6 @@
     <t>Tx_BuildingAddress</t>
   </si>
   <si>
-    <t>1280 Springfield</t>
-  </si>
-  <si>
-    <t>15 South Street</t>
-  </si>
-  <si>
-    <t>36 South Street</t>
-  </si>
-  <si>
     <t>Lease Execution Date</t>
   </si>
   <si>
@@ -143,7 +137,7 @@
     <t>Premises</t>
   </si>
   <si>
-    <t>One (1) Ground Floor Retail (hereinafter collectively referred to as “the store”) in a commercial building (hereinafter referred to as “the building”)</t>
+    <t>One (1) Ground Floor Retail (hereinafter collectively referred to as “the store”) in a commercial building (hereinafter referred to as “the building”</t>
   </si>
   <si>
     <t>Tx_Premises</t>
@@ -705,19 +699,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="70" customWidth="1"/>
-    <col min="5" max="5" width="9" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="34" customWidth="1"/>
     <col min="7" max="7" width="13" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -769,619 +764,697 @@
       <c r="Q1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" t="b">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
         <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
       </c>
       <c r="G2" t="s">
         <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" t="s">
+      <c r="I2">
+        <v>1280</v>
+      </c>
+      <c r="J2">
+        <v>36</v>
+      </c>
+      <c r="K2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>23</v>
       </c>
-      <c r="K2" t="s">
+      <c r="D3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="b">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
         <v>25</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
         <v>26</v>
       </c>
-      <c r="E3" t="b">
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" t="b">
         <v>0</v>
       </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" t="s">
         <v>28</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
         <v>29</v>
       </c>
-      <c r="E4" t="b">
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" t="b">
         <v>0</v>
       </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
         <v>32</v>
       </c>
-      <c r="E5" t="b">
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" t="b">
         <v>0</v>
       </c>
-      <c r="F5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="G12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>38</v>
       </c>
-      <c r="E7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" t="b">
-        <v>1</v>
-      </c>
-      <c r="C10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" t="b">
-        <v>1</v>
-      </c>
-      <c r="C11" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" t="s">
-        <v>52</v>
-      </c>
-      <c r="G11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" t="b">
-        <v>1</v>
-      </c>
-      <c r="C12" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="B13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
         <v>55</v>
       </c>
-      <c r="E12" t="b">
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" t="b">
         <v>0</v>
       </c>
-      <c r="F12" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="G13" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" t="s">
         <v>57</v>
       </c>
-      <c r="D13" t="s">
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
         <v>58</v>
       </c>
-      <c r="E13" t="b">
+      <c r="D14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" t="s">
+        <v>64</v>
+      </c>
+      <c r="H15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" t="b">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16" t="b">
         <v>0</v>
       </c>
-      <c r="F13" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" t="s">
-        <v>61</v>
-      </c>
-      <c r="E14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" t="s">
-        <v>62</v>
-      </c>
-      <c r="G14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="G16" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="b">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>69</v>
+      </c>
+      <c r="D17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="s">
         <v>64</v>
       </c>
-      <c r="D15" t="s">
-        <v>65</v>
-      </c>
-      <c r="E15" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" t="s">
-        <v>66</v>
-      </c>
-      <c r="G15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" t="b">
-        <v>1</v>
-      </c>
-      <c r="C16" t="s">
-        <v>68</v>
-      </c>
-      <c r="D16" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" t="b">
+      <c r="H17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" t="b">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" t="b">
         <v>0</v>
       </c>
-      <c r="F16" t="s">
-        <v>20</v>
-      </c>
-      <c r="G16" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C17" t="s">
-        <v>71</v>
-      </c>
-      <c r="D17" t="s">
-        <v>72</v>
-      </c>
-      <c r="E17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" t="s">
-        <v>66</v>
-      </c>
-      <c r="G17" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18" t="b">
-        <v>1</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="G18" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" t="s">
         <v>74</v>
       </c>
-      <c r="D18" t="s">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="b">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
         <v>75</v>
       </c>
-      <c r="E18" t="b">
+      <c r="D19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" t="s">
+        <v>64</v>
+      </c>
+      <c r="H19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="b">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" t="b">
+        <v>1</v>
+      </c>
+      <c r="G20" t="s">
+        <v>64</v>
+      </c>
+      <c r="H20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" t="b">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" t="b">
+        <v>1</v>
+      </c>
+      <c r="G21" t="s">
+        <v>83</v>
+      </c>
+      <c r="H21" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" t="s">
+        <v>86</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" t="b">
+        <v>1</v>
+      </c>
+      <c r="G22" t="s">
+        <v>87</v>
+      </c>
+      <c r="H22" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" t="s">
+        <v>90</v>
+      </c>
+      <c r="E23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23" t="b">
         <v>0</v>
       </c>
-      <c r="F18" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" t="b">
-        <v>1</v>
-      </c>
-      <c r="C19" t="s">
-        <v>77</v>
-      </c>
-      <c r="D19" t="s">
-        <v>78</v>
-      </c>
-      <c r="E19" t="b">
-        <v>1</v>
-      </c>
-      <c r="F19" t="s">
-        <v>66</v>
-      </c>
-      <c r="G19" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" t="b">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" t="s">
-        <v>81</v>
-      </c>
-      <c r="E20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F20" t="s">
-        <v>66</v>
-      </c>
-      <c r="G20" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="b">
-        <v>1</v>
-      </c>
-      <c r="C21" t="s">
-        <v>83</v>
-      </c>
-      <c r="D21" t="s">
-        <v>84</v>
-      </c>
-      <c r="E21" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" t="s">
-        <v>85</v>
-      </c>
-      <c r="G21" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" t="b">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
-        <v>87</v>
-      </c>
-      <c r="D22" t="s">
-        <v>88</v>
-      </c>
-      <c r="E22" t="b">
-        <v>1</v>
-      </c>
-      <c r="F22" t="s">
-        <v>89</v>
-      </c>
-      <c r="G22" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="G23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H23" t="s">
         <v>91</v>
       </c>
-      <c r="D23" t="s">
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" t="b">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
         <v>92</v>
       </c>
-      <c r="E23" t="b">
-        <v>0</v>
-      </c>
-      <c r="F23" t="s">
-        <v>20</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="D24" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" t="b">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="E24" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" t="b">
+        <v>1</v>
+      </c>
+      <c r="G24" t="s">
         <v>94</v>
       </c>
-      <c r="D24" t="s">
+      <c r="H24" t="s">
         <v>95</v>
       </c>
-      <c r="E24" t="b">
-        <v>1</v>
-      </c>
-      <c r="F24" t="s">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" t="b">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
         <v>96</v>
       </c>
-      <c r="G24" t="s">
+      <c r="D25" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>40</v>
-      </c>
-      <c r="B25" t="b">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="E25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" t="s">
         <v>98</v>
       </c>
-      <c r="D25" t="s">
+      <c r="H25" t="s">
         <v>99</v>
       </c>
-      <c r="E25" t="b">
-        <v>1</v>
-      </c>
-      <c r="F25" t="s">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" t="b">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
         <v>100</v>
       </c>
-      <c r="G25" t="s">
+      <c r="D26" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>40</v>
-      </c>
-      <c r="B26" t="b">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="E26" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" t="b">
+        <v>1</v>
+      </c>
+      <c r="G26" t="s">
         <v>102</v>
       </c>
-      <c r="D26" t="s">
+      <c r="H26" t="s">
         <v>103</v>
       </c>
-      <c r="E26" t="b">
-        <v>1</v>
-      </c>
-      <c r="F26" t="s">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" t="b">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
         <v>104</v>
       </c>
-      <c r="G26" t="s">
+      <c r="D27" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>40</v>
-      </c>
-      <c r="B27" t="b">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="E27" t="s">
+        <v>3</v>
+      </c>
+      <c r="F27" t="b">
+        <v>1</v>
+      </c>
+      <c r="G27" t="s">
         <v>106</v>
       </c>
-      <c r="D27" t="s">
+      <c r="H27" t="s">
         <v>107</v>
       </c>
-      <c r="E27" t="b">
-        <v>1</v>
-      </c>
-      <c r="F27" t="s">
-        <v>108</v>
-      </c>
-      <c r="G27" t="s">
-        <v>109</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q27" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R27" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dashboard update Fri 07/31/2026 22:01
</commit_message>
<xml_diff>
--- a/data/Lease Builder/MSP_Key_Provisions Template.xlsx
+++ b/data/Lease Builder/MSP_Key_Provisions Template.xlsx
@@ -8,35 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\Lease Builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DAEA0EB6-AE14-4804-AD50-51B6B577DF0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B149B4-444F-433C-9D96-BAE737F9B287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7410" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6630" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Key Provisions" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Key Provisions'!$A$1:$Q$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Key Provisions'!$A$1:$Q$33</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="122">
   <si>
     <t>Group</t>
   </si>
@@ -95,7 +82,7 @@
     <t>Property</t>
   </si>
   <si>
-    <t>15</t>
+    <t>114 Central Ave (also known as 102-104 Quimby St), Westfield, NJ 07090</t>
   </si>
   <si>
     <t>Section 1 — Premises</t>
@@ -104,10 +91,7 @@
     <t>Tx_BuildingAddress</t>
   </si>
   <si>
-    <t>1280</t>
-  </si>
-  <si>
-    <t>36</t>
+    <t>Optional</t>
   </si>
   <si>
     <t>Lease Execution Date</t>
@@ -140,7 +124,7 @@
     <t>Premises</t>
   </si>
   <si>
-    <t>One (1) Ground Floor Retail (hereinafter collectively referred to as “the store”) in a commercial building (hereinafter referred to as “the building”</t>
+    <t>One (1) Ground Floor Retail (hereinafter collectively referred to as “the store”) in a commercial building (hereinafter referred to as “the building”)</t>
   </si>
   <si>
     <t>Tx_Premises</t>
@@ -155,9 +139,6 @@
     <t>Tx_Sqft</t>
   </si>
   <si>
-    <t>Optional</t>
-  </si>
-  <si>
     <t>Tenant Share of Property</t>
   </si>
   <si>
@@ -200,9 +181,6 @@
     <t>Landlord Contact</t>
   </si>
   <si>
-    <t>jason.forster@proventusproperties.com</t>
-  </si>
-  <si>
     <t>Tx_LandlordContact</t>
   </si>
   <si>
@@ -363,16 +341,72 @@
   </si>
   <si>
     <t>Tx_LandlordContFitUp</t>
+  </si>
+  <si>
+    <t>Delivery Deadline Breach Opt</t>
+  </si>
+  <si>
+    <t>Tx_DeliveryDeadlineBreachOpt</t>
+  </si>
+  <si>
+    <t>Inspection Per</t>
+  </si>
+  <si>
+    <t>Tx_InspectionPer</t>
+  </si>
+  <si>
+    <t>Parking</t>
+  </si>
+  <si>
+    <t>Tx_Parking</t>
+  </si>
+  <si>
+    <t>Landlord Work</t>
+  </si>
+  <si>
+    <t>Tx_LandlordWork</t>
+  </si>
+  <si>
+    <t>Base Rent</t>
+  </si>
+  <si>
+    <t>Tx_BaseRent</t>
+  </si>
+  <si>
+    <t>Exhibit Tenant Work</t>
+  </si>
+  <si>
+    <t>Tx_ExhibitTenantWork</t>
+  </si>
+  <si>
+    <t>1280 Springfield</t>
+  </si>
+  <si>
+    <t>15 South Street</t>
+  </si>
+  <si>
+    <t>36 South Streed</t>
+  </si>
+  <si>
+    <t>JasonForster^Proventus^jason.forster@proventusproperties.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -395,13 +429,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -702,7 +747,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -712,6 +757,7 @@
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="6" max="6" width="34" customWidth="1"/>
     <col min="7" max="7" width="13" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="70" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -767,7 +813,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -777,50 +823,71 @@
       <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="H2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+    </row>
+    <row r="3" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>23</v>
       </c>
-      <c r="J2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="b">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>26</v>
-      </c>
+      <c r="H3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -830,20 +897,32 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>29</v>
-      </c>
+      <c r="H4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -853,22 +932,34 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="H5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -876,20 +967,32 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" t="s">
-        <v>35</v>
-      </c>
+      <c r="H6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -899,91 +1002,139 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="H7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="G8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B8" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+    </row>
+    <row r="9" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
         <v>41</v>
       </c>
-      <c r="E8" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="D9" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+    </row>
+    <row r="10" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
         <v>44</v>
       </c>
-      <c r="E9" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="D10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" t="b">
-        <v>1</v>
-      </c>
-      <c r="C10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+    </row>
+    <row r="11" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -991,68 +1142,104 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D11" t="s">
+      <c r="G11" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E11" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="H11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
+    </row>
+    <row r="12" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
         <v>51</v>
       </c>
-      <c r="G11" t="s">
+      <c r="D12" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E12" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" t="b">
-        <v>1</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="H12" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
+    </row>
+    <row r="13" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
         <v>53</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D13" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E12" t="b">
+      <c r="E13" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G13" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" t="s">
-        <v>56</v>
-      </c>
-      <c r="D13" t="s">
-        <v>57</v>
-      </c>
-      <c r="E13" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="H13" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1"/>
+    </row>
+    <row r="14" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1060,22 +1247,34 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D14" t="s">
-        <v>60</v>
-      </c>
-      <c r="E14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" t="s">
-        <v>61</v>
-      </c>
-      <c r="G14" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="H14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+    </row>
+    <row r="15" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1083,45 +1282,69 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D15" t="s">
+      <c r="H15" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+    </row>
+    <row r="16" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="b">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
         <v>64</v>
       </c>
-      <c r="E15" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="D16" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="G15" t="s">
+      <c r="E16" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" t="b">
-        <v>1</v>
-      </c>
-      <c r="C16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D16" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16" t="s">
-        <v>20</v>
-      </c>
-      <c r="G16" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+    </row>
+    <row r="17" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1129,45 +1352,69 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+    </row>
+    <row r="18" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" t="b">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
         <v>70</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D18" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" t="s">
-        <v>65</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="E18" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" t="b">
-        <v>1</v>
-      </c>
-      <c r="C18" t="s">
-        <v>73</v>
-      </c>
-      <c r="D18" t="s">
-        <v>74</v>
-      </c>
-      <c r="E18" t="b">
-        <v>0</v>
-      </c>
-      <c r="F18" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
+    </row>
+    <row r="19" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1175,22 +1422,34 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
-      </c>
-      <c r="D19" t="s">
-        <v>77</v>
-      </c>
-      <c r="E19" t="b">
-        <v>1</v>
-      </c>
-      <c r="F19" t="s">
-        <v>65</v>
-      </c>
-      <c r="G19" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="1"/>
+    </row>
+    <row r="20" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1198,184 +1457,470 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
+    </row>
+    <row r="21" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="b">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
         <v>79</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D21" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="E20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F20" t="s">
-        <v>65</v>
-      </c>
-      <c r="G20" t="s">
+      <c r="E21" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>39</v>
-      </c>
-      <c r="B21" t="b">
-        <v>1</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="G21" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D21" t="s">
+      <c r="H21" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1"/>
+    </row>
+    <row r="22" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
         <v>83</v>
       </c>
-      <c r="E21" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="D22" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="G21" t="s">
+      <c r="E22" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>39</v>
-      </c>
-      <c r="B22" t="b">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="G22" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D22" t="s">
+      <c r="H22" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1"/>
+    </row>
+    <row r="23" spans="1:17" ht="150" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
         <v>87</v>
       </c>
-      <c r="E22" t="b">
-        <v>1</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="D23" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="G22" t="s">
+      <c r="E23" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="H23" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+    </row>
+    <row r="24" spans="1:17" ht="105" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" t="b">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
         <v>90</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D24" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E23" t="b">
+      <c r="E24" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+    </row>
+    <row r="25" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" t="b">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E25" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" t="b">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>98</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+    </row>
+    <row r="27" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" t="b">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>102</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E27" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+    </row>
+    <row r="28" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" t="b">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>106</v>
+      </c>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F28" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G23" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" t="b">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s">
-        <v>93</v>
-      </c>
-      <c r="D24" t="s">
-        <v>94</v>
-      </c>
-      <c r="E24" t="b">
-        <v>1</v>
-      </c>
-      <c r="F24" t="s">
-        <v>95</v>
-      </c>
-      <c r="G24" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>39</v>
-      </c>
-      <c r="B25" t="b">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
-        <v>97</v>
-      </c>
-      <c r="D25" t="s">
-        <v>98</v>
-      </c>
-      <c r="E25" t="b">
-        <v>1</v>
-      </c>
-      <c r="F25" t="s">
-        <v>99</v>
-      </c>
-      <c r="G25" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26" t="b">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
-        <v>101</v>
-      </c>
-      <c r="D26" t="s">
-        <v>102</v>
-      </c>
-      <c r="E26" t="b">
-        <v>1</v>
-      </c>
-      <c r="F26" t="s">
-        <v>103</v>
-      </c>
-      <c r="G26" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" t="b">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s">
-        <v>105</v>
-      </c>
-      <c r="D27" t="s">
-        <v>106</v>
-      </c>
-      <c r="E27" t="b">
-        <v>1</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G28" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+    </row>
+    <row r="29" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" t="b">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
         <v>108</v>
       </c>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" t="b">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+    </row>
+    <row r="31" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" t="b">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>112</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" t="b">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>114</v>
+      </c>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+    </row>
+    <row r="33" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33" t="b">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>116</v>
+      </c>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q27" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:Q33" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="D12" r:id="rId1" xr:uid="{0CDBCC07-6A66-49FE-A738-251A84A885A6}"/>
+    <hyperlink ref="H12" r:id="rId2" xr:uid="{85817EE5-2361-41A7-8401-FE4E622443FA}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dashboard update Sat 08/01/2026  5:31
</commit_message>
<xml_diff>
--- a/data/Lease Builder/MSP_Key_Provisions Template.xlsx
+++ b/data/Lease Builder/MSP_Key_Provisions Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\Lease Builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B149B4-444F-433C-9D96-BAE737F9B287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FE27FB-F2A6-4509-A123-448C42CA8E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6630" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7410" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Key Provisions" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Key Provisions'!$A$1:$Q$33</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -750,14 +763,18 @@
   <dimension ref="A1:Q33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="70" customWidth="1"/>
-    <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="34" customWidth="1"/>
-    <col min="7" max="7" width="13" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="70" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="69.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.85546875" customWidth="1"/>
+    <col min="8" max="8" width="69.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dashboard update Sat 08/01/2026  9:04
</commit_message>
<xml_diff>
--- a/data/Lease Builder/MSP_Key_Provisions Template.xlsx
+++ b/data/Lease Builder/MSP_Key_Provisions Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\Lease Builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FE27FB-F2A6-4509-A123-448C42CA8E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C434118-40B1-40D9-822F-68E2F7CDFB70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7410" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="2730" windowWidth="47115" windowHeight="29670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Key Provisions" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="124">
   <si>
     <t>Group</t>
   </si>
@@ -402,6 +402,12 @@
   </si>
   <si>
     <t>JasonForster^Proventus^jason.forster@proventusproperties.com</t>
+  </si>
+  <si>
+    <t>There is parking behind the building which may be used by customers and invitees of the tenant on a non-exclusive basis (Attached Exhibit “E”). Landlord reserves the right to designate up to 10 parking spots for a specific tenant should it choose. Landlord and Tenant acknowledge that there is an access easement on the leased property through the ingress and egress driveways that allows the adjacent property visitors (44 South Street) to park in 4 designated parking spots along the South/East property line as per the attached site plan that will not change the current amount of parking spots designated to this building; see additional details below (#Parking)</t>
+  </si>
+  <si>
+    <t>There is parking behind the building which may be used by customers and invitees of the tenant on a non-exclusive basis (Attached Exhibit “E”). Tenant agrees no construction vans, trucks or oversized vehicles will be parked during the day or night in the lot.  Landloard reserves the right ot provide reserved parking for the office tenants and/or any of the residential apartments located in the the Building.  Consisten with stated policy within the township where the Premises are located, Tenat agrees it will make their employees aware and encourage the use of public trnasportation to get to and from work to avoid overcrowding the exiting parking lot.</t>
   </si>
 </sst>
 </file>
@@ -771,7 +777,7 @@
     <col min="6" max="6" width="32.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29.85546875" customWidth="1"/>
     <col min="8" max="8" width="69.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.28515625" customWidth="1"/>
     <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -830,7 +836,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -871,7 +877,7 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
     </row>
-    <row r="3" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1046,7 +1052,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1081,7 +1087,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1116,7 +1122,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1186,7 +1192,7 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1221,7 +1227,7 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1466,7 +1472,7 @@
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
     </row>
-    <row r="20" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1746,7 +1752,7 @@
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
     </row>
-    <row r="28" spans="1:17" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -1777,7 +1783,7 @@
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
     </row>
-    <row r="29" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>22</v>
       </c>
@@ -1808,7 +1814,7 @@
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" ht="180" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -1828,8 +1834,12 @@
       <c r="G30" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
+      <c r="H30" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>123</v>
+      </c>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
@@ -1839,7 +1849,7 @@
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
     </row>
-    <row r="31" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>22</v>
       </c>
@@ -1901,7 +1911,7 @@
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
     </row>
-    <row r="33" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>22</v>
       </c>

</xml_diff>